<commit_message>
Replace template data with clean dummy sample rows
Remove the real-looking patient record; ship two clearly-fictional
sample patients demonstrating the grouping rule and Procedures format.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ChargePilot-Template.xlsx
+++ b/ChargePilot-Template.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -567,17 +567,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Sample</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>1/15/1980</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -585,34 +585,36 @@
           <t>M</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>123 Main Street</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>62704</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Aetna</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>123456789</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -622,64 +624,61 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1/1/2026</t>
+          <t>1/5/2026</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>LOZANO, MATTHEW</t>
+          <t>DOE, JANE</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>AUTH5521093</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
+          <t>AUTH100001</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>80053*1*59*I10,Z00.00 ; 80061*2**E11.9,E78.5</t>
-        </is>
-      </c>
+          <t>99213*1**J06.9 ; 80053*1*59*E11.9,I10</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Sample</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>1/15/1980</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -687,34 +686,36 @@
           <t>M</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>123 Main Street</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>62704</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Aetna</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>123456789</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -724,49 +725,57 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1/2/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>12D3456789</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>85025*1**I10 ; 83036*1*26*E11.9 ; 84443*1**E03.9</t>
-        </is>
-      </c>
+          <t>85025*1**I10 ; 83036*1*26*E11.9</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Sample</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>1/15/1980</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -774,34 +783,36 @@
           <t>M</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>123 Main Street</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>IL</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>62704</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Aetna</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>123456789</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -811,94 +822,94 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1/5/2026</t>
+          <t>1/12/2026</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>LOZANO, MATTHEW</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>AUTH100001</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>87798*3*qw*J06.9,K21.9 ; 87500*1**N39.0</t>
-        </is>
-      </c>
+          <t>80061*1**E78.5,Z00.00</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>6/22/1975</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>456 Oak Avenue</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>WI</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>53703</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Blue Cross Blue Shield</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>987654321</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -913,89 +924,89 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>AUTH5521093</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>DOE, JANE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>80307*2*26*I10 ; 81225*1**E11.9 ; 82306*1**E78.5</t>
-        </is>
-      </c>
+          <t>99214*1*25*Z00.00 ; 84443*1**E03.9</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>6/22/1975</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>456 Oak Avenue</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>WI</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>53703</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Blue Cross Blue Shield</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>987654321</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1005,94 +1016,94 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>1/7/2026</t>
+          <t>1/9/2026</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>LOZANO, MATTHEW</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>AUTH5521093</t>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>12D3456789</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>85025*1**I10,F32.9 ; 87651*2*tc*J06.9</t>
-        </is>
-      </c>
+          <t>87798*2*qw*J06.9</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Demo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10/30/1945</t>
+          <t>6/22/1975</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>457 REGINA DR</t>
+          <t>456 Oak Avenue</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PAINESVILLE</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>WI</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>44077</t>
+          <t>53703</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>United HealthCare</t>
+          <t>Blue Cross Blue Shield</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>930907430</t>
+          <t>987654321</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1102,422 +1113,42 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/13/2026</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1083325641</t>
+          <t>1234567890</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1083325641</t>
-        </is>
-      </c>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>AUTH200002</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>83735*1**E03.9 ; 82607*1**N39.0 ; 84443*1**K21.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>10/30/1945</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>457 REGINA DR</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>PAINESVILLE</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>44077</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>United HealthCare</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>930907430</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>1/1/2026</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>1/9/2026</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>LOZANO, MATTHEW</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>AUTH5521093</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>87502*1**J06.9 ; 87506*2*59*R10.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>10/30/1945</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>457 REGINA DR</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>PAINESVILLE</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>44077</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>United HealthCare</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>930907430</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>1/1/2026</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>1/12/2026</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>80061*1**E78.5,M54.50 ; 81200*1**E11.9 ; 99999*1**I10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>10/30/1945</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>457 REGINA DR</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>PAINESVILLE</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>44077</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>United HealthCare</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>930907430</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>1/1/2026</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1/13/2026</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>LOZANO, MATTHEW</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>81256*2**F41.9 ; 81260*1*26*I10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>10/30/1945</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>457 REGINA DR</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>PAINESVILLE</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>44077</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>United HealthCare</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>930907430</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>1/1/2026</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1/14/2026</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>1083325641</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>LOZANO, MATTHEW</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>AUTH5521093</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>34D2098612</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>85025*1**I10 ; 80053*1**Z00.00 ; 87798*4*qw*J06.9</t>
-        </is>
-      </c>
+          <t>80307*1*26*F11.20</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>